<commit_message>
feat: implement certificate styling and add necessary assets for document generation
</commit_message>
<xml_diff>
--- a/admin data/certificate_downloads.xlsx
+++ b/admin data/certificate_downloads.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F2"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -432,225 +432,25 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>Dr. Madhuri Revanwar</v>
+        <v>Dr. Anita Sharma</v>
       </c>
       <c r="C2" t="str">
-        <v>sd</v>
+        <v>asx</v>
       </c>
       <c r="D2" t="str">
-        <v>ICAR-Agricultural Technology Application Research Institute, Zone I, Ludhiana</v>
+        <v>ICAR-Agricultural Technology Application Research Institute, Zone IV, Patna</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-07-28 23:13:54</v>
+        <v>2026-07-29 10:50:10</v>
       </c>
       <c r="F2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Mrs. Kavita Deshpande</v>
-      </c>
-      <c r="C3" t="str">
-        <v>CSA</v>
-      </c>
-      <c r="D3" t="str">
-        <v>ICAR-Agricultural Technology Application Research Institute, Zone IX, Jabalpur</v>
-      </c>
-      <c r="E3" t="str">
-        <v>2026-07-28 23:14:09</v>
-      </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Dr. Madhuri Revanwar</v>
-      </c>
-      <c r="C4" t="str">
-        <v>ASFFA</v>
-      </c>
-      <c r="D4" t="str">
-        <v>ICAR-Agricultural Technology Application Research Institute, Zone V, Kolkata</v>
-      </c>
-      <c r="E4" t="str">
-        <v>2026-07-28 23:15:02</v>
-      </c>
-      <c r="F4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Dr. Madhuri Revanwar</v>
-      </c>
-      <c r="C5" t="str">
-        <v>KVK, Nanded-II</v>
-      </c>
-      <c r="D5" t="str">
-        <v>ICAR-Agricultural Technology Application Research Institute, Zone VIII, Pune</v>
-      </c>
-      <c r="E5" t="str">
-        <v>2026-07-28 23:44:45</v>
-      </c>
-      <c r="F5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Dr. Priya Patel</v>
-      </c>
-      <c r="C6" t="str">
-        <v>daf</v>
-      </c>
-      <c r="D6" t="str">
-        <v>ICAR-Agricultural Technology Application Research Institute, Zone II, Jodhpur</v>
-      </c>
-      <c r="E6" t="str">
-        <v>2026-07-28 23:58:03</v>
-      </c>
-      <c r="F6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Mr. Anita Sharma</v>
-      </c>
-      <c r="C7" t="str">
-        <v>fsg</v>
-      </c>
-      <c r="D7" t="str">
-        <v>ICAR-Agricultural Technology Application Research Institute, Zone IX, Jabalpur</v>
-      </c>
-      <c r="E7" t="str">
-        <v>2026-07-29 00:19:49</v>
-      </c>
-      <c r="F7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Mr. Priya Patel</v>
-      </c>
-      <c r="C8" t="str">
-        <v>DS</v>
-      </c>
-      <c r="D8" t="str">
-        <v>ICAR-Agricultural Technology Application Research Institute, Zone II, Jodhpur</v>
-      </c>
-      <c r="E8" t="str">
-        <v>2026-07-29 00:32:38</v>
-      </c>
-      <c r="F8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Mr. Kavita Deshpande</v>
-      </c>
-      <c r="C9" t="str">
-        <v>DSfqeqre</v>
-      </c>
-      <c r="D9" t="str">
-        <v>ICAR-Agricultural Technology Application Research Institute, Zone IV, Patna</v>
-      </c>
-      <c r="E9" t="str">
-        <v>2026-07-29 00:33:34</v>
-      </c>
-      <c r="F9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Mr. Kavita Deshpande</v>
-      </c>
-      <c r="C10" t="str">
-        <v>sacadGQRWGRRWTRW</v>
-      </c>
-      <c r="D10" t="str">
-        <v>ICAR-Agricultural Technology Application Research Institute, Zone X, Hyderabad</v>
-      </c>
-      <c r="E10" t="str">
-        <v>2026-07-29 00:41:20</v>
-      </c>
-      <c r="F10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Mr. Venkatesh Rao</v>
-      </c>
-      <c r="C11" t="str">
-        <v>ascacs</v>
-      </c>
-      <c r="D11" t="str">
-        <v>ICAR-Agricultural Technology Application Research Institute, Zone II, Jodhpur</v>
-      </c>
-      <c r="E11" t="str">
-        <v>2026-07-29 00:47:35</v>
-      </c>
-      <c r="F11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" t="str">
-        <v>Mrs. Priya Patel</v>
-      </c>
-      <c r="C12" t="str">
-        <v>acdadd</v>
-      </c>
-      <c r="D12" t="str">
-        <v>ICAR-Agricultural Technology Application Research Institute, Zone II, Jodhpur</v>
-      </c>
-      <c r="E12" t="str">
-        <v>2026-07-29 01:19:34</v>
-      </c>
-      <c r="F12">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <sheetProtection sheet="1" selectLockedCells="1" selectUnlockedCells="1" password="D9A6"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: remove unused lightningcss dependencies and add certificate downloads data file
</commit_message>
<xml_diff>
--- a/admin data/certificate_downloads.xlsx
+++ b/admin data/certificate_downloads.xlsx
@@ -432,16 +432,16 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>Dr. Anita Sharma</v>
+        <v>Mr. Madhuri Revanwar</v>
       </c>
       <c r="C2" t="str">
-        <v>asx</v>
+        <v>wqdef</v>
       </c>
       <c r="D2" t="str">
-        <v>ICAR-Agricultural Technology Application Research Institute, Zone IV, Patna</v>
+        <v>ICAR-Agricultural Technology Application Research Institute, Zone I, Ludhiana</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-07-29 10:50:10</v>
+        <v>2026-07-29 10:59:34</v>
       </c>
       <c r="F2">
         <v>1</v>

</xml_diff>